<commit_message>
UI improvements: calculator navigation, dark mode styling, banner adjustments
</commit_message>
<xml_diff>
--- a/static/investment_results.xlsx
+++ b/static/investment_results.xlsx
@@ -436,7 +436,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -449,7 +449,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -462,7 +462,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -475,7 +475,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -488,7 +488,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -501,7 +501,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -514,7 +514,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -527,7 +527,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -540,7 +540,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-11-11</t>
+          <t>2026-11-12</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -553,7 +553,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-12</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -566,7 +566,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2027-01-11</t>
+          <t>2027-01-12</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -579,7 +579,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2027-02-11</t>
+          <t>2027-02-12</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -592,7 +592,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2027-03-11</t>
+          <t>2027-03-12</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -605,7 +605,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2027-04-11</t>
+          <t>2027-04-12</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -618,7 +618,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2027-05-11</t>
+          <t>2027-05-12</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -631,7 +631,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2027-06-11</t>
+          <t>2027-06-12</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -644,7 +644,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2027-07-11</t>
+          <t>2027-07-12</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -657,7 +657,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2027-08-11</t>
+          <t>2027-08-12</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -670,7 +670,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2027-09-11</t>
+          <t>2027-09-12</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -683,7 +683,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2027-10-11</t>
+          <t>2027-10-12</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -696,7 +696,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2027-11-11</t>
+          <t>2027-11-12</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -709,7 +709,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2027-12-11</t>
+          <t>2027-12-12</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -722,7 +722,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2028-01-11</t>
+          <t>2028-01-12</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -735,7 +735,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2028-02-11</t>
+          <t>2028-02-12</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -748,7 +748,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2028-03-11</t>
+          <t>2028-03-12</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -761,7 +761,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2028-04-11</t>
+          <t>2028-04-12</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -774,7 +774,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2028-05-11</t>
+          <t>2028-05-12</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -787,7 +787,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2028-06-11</t>
+          <t>2028-06-12</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -800,7 +800,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2028-07-11</t>
+          <t>2028-07-12</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -813,7 +813,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2028-08-11</t>
+          <t>2028-08-12</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -826,7 +826,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2028-09-11</t>
+          <t>2028-09-12</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -839,7 +839,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2028-10-11</t>
+          <t>2028-10-12</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -852,7 +852,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2028-11-11</t>
+          <t>2028-11-12</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -865,7 +865,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2028-12-11</t>
+          <t>2028-12-12</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -878,7 +878,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2029-01-11</t>
+          <t>2029-01-12</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -891,7 +891,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2029-02-11</t>
+          <t>2029-02-12</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -904,7 +904,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2029-03-11</t>
+          <t>2029-03-12</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -917,7 +917,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2029-04-11</t>
+          <t>2029-04-12</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -930,7 +930,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2029-05-11</t>
+          <t>2029-05-12</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -943,7 +943,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2029-06-11</t>
+          <t>2029-06-12</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -956,7 +956,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2029-07-11</t>
+          <t>2029-07-12</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -969,7 +969,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2029-08-11</t>
+          <t>2029-08-12</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -982,7 +982,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2029-09-11</t>
+          <t>2029-09-12</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -995,7 +995,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2029-10-11</t>
+          <t>2029-10-12</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1008,7 +1008,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2029-11-11</t>
+          <t>2029-11-12</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1021,7 +1021,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2029-12-11</t>
+          <t>2029-12-12</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1034,7 +1034,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2030-01-11</t>
+          <t>2030-01-12</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1047,7 +1047,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2030-02-11</t>
+          <t>2030-02-12</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1060,7 +1060,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2030-03-11</t>
+          <t>2030-03-12</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1073,7 +1073,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2030-04-11</t>
+          <t>2030-04-12</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1086,7 +1086,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2030-05-11</t>
+          <t>2030-05-12</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1099,7 +1099,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2030-06-11</t>
+          <t>2030-06-12</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1112,7 +1112,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2030-07-11</t>
+          <t>2030-07-12</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1125,7 +1125,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2030-08-11</t>
+          <t>2030-08-12</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1138,7 +1138,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2030-09-11</t>
+          <t>2030-09-12</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1151,7 +1151,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2030-10-11</t>
+          <t>2030-10-12</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1164,7 +1164,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2030-11-11</t>
+          <t>2030-11-12</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1177,7 +1177,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2030-12-11</t>
+          <t>2030-12-12</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1190,7 +1190,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2031-01-11</t>
+          <t>2031-01-12</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1203,7 +1203,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2031-02-11</t>
+          <t>2031-02-12</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1216,7 +1216,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2031-03-11</t>
+          <t>2031-03-12</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1229,7 +1229,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2031-04-11</t>
+          <t>2031-04-12</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1242,7 +1242,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2031-05-11</t>
+          <t>2031-05-12</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1255,7 +1255,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2031-06-11</t>
+          <t>2031-06-12</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1268,7 +1268,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2031-07-11</t>
+          <t>2031-07-12</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1281,7 +1281,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2031-08-11</t>
+          <t>2031-08-12</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1294,7 +1294,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2031-09-11</t>
+          <t>2031-09-12</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1307,7 +1307,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2031-10-11</t>
+          <t>2031-10-12</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1320,7 +1320,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2031-11-11</t>
+          <t>2031-11-12</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1333,7 +1333,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2031-12-11</t>
+          <t>2031-12-12</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1346,7 +1346,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2032-01-11</t>
+          <t>2032-01-12</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1359,7 +1359,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2032-02-11</t>
+          <t>2032-02-12</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1372,7 +1372,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2032-03-11</t>
+          <t>2032-03-12</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1385,7 +1385,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2032-04-11</t>
+          <t>2032-04-12</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1398,7 +1398,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2032-05-11</t>
+          <t>2032-05-12</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1411,7 +1411,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2032-06-11</t>
+          <t>2032-06-12</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1424,7 +1424,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2032-07-11</t>
+          <t>2032-07-12</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1437,7 +1437,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2032-08-11</t>
+          <t>2032-08-12</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1450,7 +1450,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2032-09-11</t>
+          <t>2032-09-12</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1463,7 +1463,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2032-10-11</t>
+          <t>2032-10-12</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1476,7 +1476,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2032-11-11</t>
+          <t>2032-11-12</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1489,7 +1489,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2032-12-11</t>
+          <t>2032-12-12</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1502,7 +1502,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2033-01-11</t>
+          <t>2033-01-12</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1515,7 +1515,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2033-02-11</t>
+          <t>2033-02-12</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1528,7 +1528,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2033-03-11</t>
+          <t>2033-03-12</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1541,7 +1541,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2033-04-11</t>
+          <t>2033-04-12</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1554,7 +1554,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2033-05-11</t>
+          <t>2033-05-12</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1567,7 +1567,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2033-06-11</t>
+          <t>2033-06-12</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1580,7 +1580,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2033-07-11</t>
+          <t>2033-07-12</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1593,7 +1593,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2033-08-11</t>
+          <t>2033-08-12</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1606,7 +1606,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2033-09-11</t>
+          <t>2033-09-12</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1619,7 +1619,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2033-10-11</t>
+          <t>2033-10-12</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1632,7 +1632,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2033-11-11</t>
+          <t>2033-11-12</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1645,7 +1645,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2033-12-11</t>
+          <t>2033-12-12</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1658,7 +1658,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2034-01-11</t>
+          <t>2034-01-12</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1671,7 +1671,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2034-02-11</t>
+          <t>2034-02-12</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1684,7 +1684,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2034-03-11</t>
+          <t>2034-03-12</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1697,7 +1697,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2034-04-11</t>
+          <t>2034-04-12</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -1710,7 +1710,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2034-05-11</t>
+          <t>2034-05-12</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -1723,7 +1723,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2034-06-11</t>
+          <t>2034-06-12</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -1736,7 +1736,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2034-07-11</t>
+          <t>2034-07-12</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -1749,7 +1749,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2034-08-11</t>
+          <t>2034-08-12</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -1762,7 +1762,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2034-09-11</t>
+          <t>2034-09-12</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -1775,7 +1775,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2034-10-11</t>
+          <t>2034-10-12</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -1788,7 +1788,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2034-11-11</t>
+          <t>2034-11-12</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -1801,7 +1801,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2034-12-11</t>
+          <t>2034-12-12</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -1814,7 +1814,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2035-01-11</t>
+          <t>2035-01-12</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -1827,7 +1827,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2035-02-11</t>
+          <t>2035-02-12</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -1840,7 +1840,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2035-03-11</t>
+          <t>2035-03-12</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -1853,7 +1853,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2035-04-11</t>
+          <t>2035-04-12</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -1866,7 +1866,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2035-05-11</t>
+          <t>2035-05-12</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -1879,7 +1879,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2035-06-11</t>
+          <t>2035-06-12</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -1892,7 +1892,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2035-07-11</t>
+          <t>2035-07-12</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -1905,7 +1905,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2035-08-11</t>
+          <t>2035-08-12</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -1918,7 +1918,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2035-09-11</t>
+          <t>2035-09-12</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -1931,7 +1931,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2035-10-11</t>
+          <t>2035-10-12</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -1944,7 +1944,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2035-11-11</t>
+          <t>2035-11-12</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -1957,7 +1957,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2035-12-11</t>
+          <t>2035-12-12</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -1970,7 +1970,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2036-01-11</t>
+          <t>2036-01-12</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -1983,7 +1983,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2036-02-11</t>
+          <t>2036-02-12</t>
         </is>
       </c>
       <c r="B121" t="n">

</xml_diff>